<commit_message>
pb 10.5.1 -d,e - lab10 - tema
</commit_message>
<xml_diff>
--- a/studentiStrategyExcel.xlsx
+++ b/studentiStrategyExcel.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="19">
   <si>
     <t>Andrei</t>
   </si>
@@ -47,16 +47,13 @@
     <t>Popescu</t>
   </si>
   <si>
-    <t>TI131/1,</t>
-  </si>
-  <si>
     <t>Maria</t>
   </si>
   <si>
     <t>Pana</t>
   </si>
   <si>
-    <t>TI131/2,</t>
+    <t>TI131/2</t>
   </si>
   <si>
     <t>Gabriela</t>
@@ -181,7 +178,7 @@
         <v>10</v>
       </c>
       <c r="D4" t="s" s="0">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="E4" t="n" s="0">
         <v>10.0</v>
@@ -192,13 +189,13 @@
         <v>1029.0</v>
       </c>
       <c r="B5" t="s" s="0">
+        <v>11</v>
+      </c>
+      <c r="C5" t="s" s="0">
         <v>12</v>
       </c>
-      <c r="C5" t="s" s="0">
-        <v>13</v>
-      </c>
       <c r="D5" t="s" s="0">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E5" t="n" s="0">
         <v>4.1</v>
@@ -209,13 +206,13 @@
         <v>1029.0</v>
       </c>
       <c r="B6" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="C6" t="s" s="0">
         <v>15</v>
       </c>
-      <c r="C6" t="s" s="0">
-        <v>16</v>
-      </c>
       <c r="D6" t="s" s="0">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E6" t="n" s="0">
         <v>7.33</v>
@@ -226,13 +223,13 @@
         <v>1029.0</v>
       </c>
       <c r="B7" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="C7" t="s" s="0">
         <v>17</v>
       </c>
-      <c r="C7" t="s" s="0">
-        <v>18</v>
-      </c>
       <c r="D7" t="s" s="0">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E7" t="n" s="0">
         <v>3.2</v>
@@ -243,13 +240,13 @@
         <v>1029.0</v>
       </c>
       <c r="B8" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="C8" t="s" s="0">
         <v>17</v>
       </c>
-      <c r="C8" t="s" s="0">
-        <v>18</v>
-      </c>
       <c r="D8" t="s" s="0">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="E8" t="n" s="0">
         <v>5.12</v>
@@ -263,10 +260,10 @@
         <v>0</v>
       </c>
       <c r="C9" t="s" s="0">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D9" t="s" s="0">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E9" t="n" s="0">
         <v>2.22</v>

</xml_diff>